<commit_message>
data logger + port gradio
</commit_message>
<xml_diff>
--- a/Test/record document/1.xlsx
+++ b/Test/record document/1.xlsx
@@ -422,11 +422,15 @@
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Mary Chan</t>
+        </is>
+      </c>
       <c r="C1" t="inlineStr"/>
       <c r="D1" t="inlineStr">
         <is>
-          <t>2025/06</t>
+          <t>2025/07</t>
         </is>
       </c>
     </row>
@@ -436,7 +440,11 @@
           <t>Birth date</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1938/3/8</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -446,7 +454,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1號床</t>
         </is>
       </c>
     </row>

</xml_diff>